<commit_message>
[EXECUTOR] Realization Class rubric v1.2 + Case_01 P2 tag wave: 46 rules realization_class T17/P23/C6 (Doc18 fields 25/26 + Anexo A/D, control_set, xlsx), blind audit 41/46 + 2 adjudicated fixes, build_control_set v1.1 — documents-only (ontology/dashboards/mirrors/KG deferred)
</commit_message>
<xml_diff>
--- a/02_CASES/Case_01_TinyTask_SaaS/02_PHASE2_RULES_RICH/12_Rules_Catalog.xlsx
+++ b/02_CASES/Case_01_TinyTask_SaaS/02_PHASE2_RULES_RICH/12_Rules_Catalog.xlsx
@@ -588,7 +588,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -728,7 +727,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
@@ -1020,7 +1018,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
@@ -1070,7 +1067,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
@@ -1143,7 +1139,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -1151,7 +1146,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -1354,7 +1348,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -1362,7 +1355,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -3448,7 +3440,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -3456,7 +3447,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -3922,7 +3912,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -3930,7 +3919,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -4582,7 +4570,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -4590,7 +4577,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -9844,7 +9830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q52"/>
+  <dimension ref="A1:S52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -9873,7 +9859,13 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>STALE UNTIL REGENERATED — banner note per the Sync rule (REALIZATION_CLASS_RUBRIC v1.1 §4, Amendment A4): realization_class / realization_class_secondary columns added 2026-09-05. The sheet's 46 rule rows match Doc18; its NI and stub columns remain as-is (pre-existing staleness not remediated).</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -9881,7 +9873,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -9968,6 +9959,16 @@
           <t>Sprint 1 Finding</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>realization_class</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>realization_class_secondary</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -10049,6 +10050,16 @@
         </is>
       </c>
       <c r="Q6" s="6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -10130,6 +10141,16 @@
         </is>
       </c>
       <c r="Q7" s="6" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -10215,6 +10236,16 @@
           <t>F-03: references phantom PO-D-01.3-001</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -10296,6 +10327,16 @@
         </is>
       </c>
       <c r="Q9" s="6" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -10377,6 +10418,16 @@
         </is>
       </c>
       <c r="Q10" s="6" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -10458,6 +10509,16 @@
         </is>
       </c>
       <c r="Q11" s="6" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -10539,6 +10600,16 @@
         </is>
       </c>
       <c r="Q12" s="6" t="inlineStr"/>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -10620,6 +10691,16 @@
         </is>
       </c>
       <c r="Q13" s="6" t="inlineStr"/>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -10701,6 +10782,16 @@
         </is>
       </c>
       <c r="Q14" s="6" t="inlineStr"/>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -10782,6 +10873,16 @@
         </is>
       </c>
       <c r="Q15" s="6" t="inlineStr"/>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -10863,6 +10964,16 @@
         </is>
       </c>
       <c r="Q16" s="6" t="inlineStr"/>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -10944,6 +11055,16 @@
         </is>
       </c>
       <c r="Q17" s="6" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -11025,6 +11146,16 @@
         </is>
       </c>
       <c r="Q18" s="6" t="inlineStr"/>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -11106,6 +11237,16 @@
         </is>
       </c>
       <c r="Q19" s="6" t="inlineStr"/>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -11187,6 +11328,16 @@
         </is>
       </c>
       <c r="Q20" s="6" t="inlineStr"/>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -11268,6 +11419,16 @@
         </is>
       </c>
       <c r="Q21" s="6" t="inlineStr"/>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -11349,6 +11510,16 @@
         </is>
       </c>
       <c r="Q22" s="6" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -11430,6 +11601,16 @@
         </is>
       </c>
       <c r="Q23" s="6" t="inlineStr"/>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -11511,6 +11692,16 @@
         </is>
       </c>
       <c r="Q24" s="6" t="inlineStr"/>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -11592,6 +11783,16 @@
         </is>
       </c>
       <c r="Q25" s="6" t="inlineStr"/>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -11673,6 +11874,16 @@
         </is>
       </c>
       <c r="Q26" s="6" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -11754,6 +11965,16 @@
         </is>
       </c>
       <c r="Q27" s="6" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -11835,6 +12056,16 @@
         </is>
       </c>
       <c r="Q28" s="6" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
@@ -11916,6 +12147,16 @@
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>CAPABILITY</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -11997,6 +12238,16 @@
         </is>
       </c>
       <c r="Q30" s="6" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>CAPABILITY</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
@@ -12078,6 +12329,16 @@
         </is>
       </c>
       <c r="Q31" s="6" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>CAPABILITY</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
@@ -12159,6 +12420,16 @@
         </is>
       </c>
       <c r="Q32" s="6" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>CAPABILITY</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
@@ -12240,6 +12511,16 @@
         </is>
       </c>
       <c r="Q33" s="6" t="inlineStr"/>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
@@ -12321,6 +12602,16 @@
         </is>
       </c>
       <c r="Q34" s="6" t="inlineStr"/>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
@@ -12402,6 +12693,16 @@
         </is>
       </c>
       <c r="Q35" s="6" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="6" t="inlineStr">
@@ -12483,6 +12784,16 @@
         </is>
       </c>
       <c r="Q36" s="6" t="inlineStr"/>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
@@ -12564,6 +12875,16 @@
         </is>
       </c>
       <c r="Q37" s="6" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
@@ -12645,6 +12966,16 @@
         </is>
       </c>
       <c r="Q38" s="6" t="inlineStr"/>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
@@ -12726,6 +13057,16 @@
         </is>
       </c>
       <c r="Q39" s="6" t="inlineStr"/>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
@@ -12807,6 +13148,16 @@
         </is>
       </c>
       <c r="Q40" s="6" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
@@ -12888,6 +13239,16 @@
         </is>
       </c>
       <c r="Q41" s="6" t="inlineStr"/>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -12969,6 +13330,16 @@
         </is>
       </c>
       <c r="Q42" s="6" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
@@ -13050,6 +13421,16 @@
         </is>
       </c>
       <c r="Q43" s="6" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>CAPABILITY</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -13131,6 +13512,16 @@
         </is>
       </c>
       <c r="Q44" s="6" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
@@ -13212,6 +13603,16 @@
         </is>
       </c>
       <c r="Q45" s="6" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -13293,6 +13694,16 @@
         </is>
       </c>
       <c r="Q46" s="6" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -13374,6 +13785,16 @@
         </is>
       </c>
       <c r="Q47" s="6" t="inlineStr"/>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -13455,6 +13876,16 @@
         </is>
       </c>
       <c r="Q48" s="6" t="inlineStr"/>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>CAPABILITY</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -13536,6 +13967,16 @@
         </is>
       </c>
       <c r="Q49" s="6" t="inlineStr"/>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
@@ -13617,6 +14058,16 @@
         </is>
       </c>
       <c r="Q50" s="6" t="inlineStr"/>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
@@ -13698,6 +14149,16 @@
         </is>
       </c>
       <c r="Q51" s="6" t="inlineStr"/>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>PROCESS</t>
+        </is>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="12" t="inlineStr">
@@ -15508,7 +15969,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -15516,7 +15976,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -16757,7 +17216,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -16765,7 +17223,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -18488,7 +18945,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -18496,7 +18952,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -18836,7 +19291,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -18844,7 +19298,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -19853,7 +20306,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -19861,7 +20313,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -20091,7 +20542,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -20099,7 +20549,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
@@ -21309,7 +21758,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -21317,7 +21765,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>

</xml_diff>